<commit_message>
Update Stage 4 outcomes and thesis guidance
</commit_message>
<xml_diff>
--- a/analysis(S4)/tables/variable_role_map.xlsx
+++ b/analysis(S4)/tables/variable_role_map.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="483" uniqueCount="129">
   <si>
     <t>variable</t>
   </si>
@@ -187,27 +187,30 @@
     <t>structural_virality_mean</t>
   </si>
   <si>
+    <t>wiener_index_mean</t>
+  </si>
+  <si>
+    <t>centrality_mean</t>
+  </si>
+  <si>
+    <t>agent_deg_centrality_mean</t>
+  </si>
+  <si>
+    <t>avg_out_degree_centrality_mean</t>
+  </si>
+  <si>
+    <t>repeat_exposure_1st_nodes_pct</t>
+  </si>
+  <si>
+    <t>repeat_exposure_2nd_nodes_pct</t>
+  </si>
+  <si>
+    <t>gender_assortativity_mean</t>
+  </si>
+  <si>
     <t>duration_mean_of_means</t>
   </si>
   <si>
-    <t>agent_deg_centrality_mean</t>
-  </si>
-  <si>
-    <t>avg_out_degree_centrality_mean</t>
-  </si>
-  <si>
-    <t>centrality_mean</t>
-  </si>
-  <si>
-    <t>repeat_exposure_1st_nodes_pct</t>
-  </si>
-  <si>
-    <t>repeat_exposure_2nd_nodes_pct</t>
-  </si>
-  <si>
-    <t>gender_assortativity_mean</t>
-  </si>
-  <si>
     <t>MatchScore_mean</t>
   </si>
   <si>
@@ -310,7 +313,7 @@
     <t>content control</t>
   </si>
   <si>
-    <t>diffusion outcome</t>
+    <t>supplementary diffusion outcome</t>
   </si>
   <si>
     <t>agent descriptor</t>
@@ -322,10 +325,7 @@
     <t>exposure/stability control</t>
   </si>
   <si>
-    <t>agent-level diffusion outcome</t>
-  </si>
-  <si>
-    <t>diffusion-pattern descriptor</t>
+    <t>agent-level supplementary diffusion outcome</t>
   </si>
   <si>
     <t>agent-topic grouping variable</t>
@@ -340,16 +340,16 @@
     <t>diagnostic flag</t>
   </si>
   <si>
-    <t>agent-topic diffusion outcome</t>
+    <t>agent-topic supplementary diffusion outcome</t>
   </si>
   <si>
     <t>Observed after posting; do not use as leakage-free predictor.</t>
   </si>
   <si>
-    <t>Aggregated observed diffusion result.</t>
-  </si>
-  <si>
-    <t>Derived from observed diffusion/network; do not interpret as an ex-ante causal predictor.</t>
+    <t>Aggregated observed diffusion result; do not use as an ordinary RHS predictor for mechanically related diffusion outcomes.</t>
+  </si>
+  <si>
+    <t>Aggregated observed diffusion result; do not use as a leakage-free predictor.</t>
   </si>
   <si>
     <t>Article-agent case identifier only.</t>
@@ -370,7 +370,7 @@
     <t>Observable article-format control.</t>
   </si>
   <si>
-    <t>Content-level diffusion performance or cascade-shape outcome.</t>
+    <t>Article-agent diffusion performance or cascade-shape outcome.</t>
   </si>
   <si>
     <t>Used for description or deriving existing S3 categories, not as high-cardinality main regression predictors.</t>
@@ -385,10 +385,7 @@
     <t>Main article-count adjustment.</t>
   </si>
   <si>
-    <t>Agent-level average diffusion pattern or capability measure.</t>
-  </si>
-  <si>
-    <t>Use only as a supplementary diagnostic or descriptive heterogeneity descriptor.</t>
+    <t>Agent-level average diffusion performance, cascade-shape, exposure, or reconstructed network-position outcome.</t>
   </si>
   <si>
     <t>Defines content-agent matching cells and controls.</t>
@@ -403,7 +400,7 @@
     <t>Sparse-cell interpretation/sensitivity flag.</t>
   </si>
   <si>
-    <t>Outcome for content-agent matching analysis.</t>
+    <t>Agent-topic average diffusion performance, cascade-shape, or reconstructed network-position outcome.</t>
   </si>
 </sst>
 </file>
@@ -735,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H81"/>
+  <dimension ref="A1:H87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:8">
@@ -769,13 +766,13 @@
         <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E2" t="b">
         <v>0</v>
@@ -792,13 +789,13 @@
         <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" t="b">
         <v>0</v>
@@ -815,13 +812,13 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D4" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E4" t="b">
         <v>0</v>
@@ -838,13 +835,13 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>
@@ -861,13 +858,13 @@
         <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E6" t="b">
         <v>0</v>
@@ -884,13 +881,13 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E7" t="b">
         <v>1</v>
@@ -907,13 +904,13 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E8" t="b">
         <v>1</v>
@@ -930,13 +927,13 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E9" t="b">
         <v>1</v>
@@ -953,13 +950,13 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D10" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E10" t="b">
         <v>1</v>
@@ -976,13 +973,13 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E11" t="b">
         <v>1</v>
@@ -999,13 +996,13 @@
         <v>18</v>
       </c>
       <c r="B12" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C12" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D12" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E12" t="b">
         <v>1</v>
@@ -1022,13 +1019,13 @@
         <v>19</v>
       </c>
       <c r="B13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D13" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E13" t="b">
         <v>1</v>
@@ -1045,13 +1042,13 @@
         <v>20</v>
       </c>
       <c r="B14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D14" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E14" t="b">
         <v>1</v>
@@ -1068,13 +1065,13 @@
         <v>21</v>
       </c>
       <c r="B15" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C15" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D15" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E15" t="b">
         <v>1</v>
@@ -1091,13 +1088,13 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D16" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E16" t="b">
         <v>1</v>
@@ -1114,13 +1111,13 @@
         <v>23</v>
       </c>
       <c r="B17" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D17" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -1137,13 +1134,13 @@
         <v>24</v>
       </c>
       <c r="B18" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C18" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D18" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E18" t="b">
         <v>1</v>
@@ -1160,13 +1157,13 @@
         <v>25</v>
       </c>
       <c r="B19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E19" t="b">
         <v>0</v>
@@ -1186,13 +1183,13 @@
         <v>26</v>
       </c>
       <c r="B20" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D20" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E20" t="b">
         <v>0</v>
@@ -1212,13 +1209,13 @@
         <v>27</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D21" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E21" t="b">
         <v>0</v>
@@ -1238,13 +1235,13 @@
         <v>28</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C22" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D22" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E22" t="b">
         <v>0</v>
@@ -1264,13 +1261,13 @@
         <v>29</v>
       </c>
       <c r="B23" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D23" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E23" t="b">
         <v>0</v>
@@ -1290,13 +1287,13 @@
         <v>30</v>
       </c>
       <c r="B24" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D24" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E24" t="b">
         <v>0</v>
@@ -1316,13 +1313,13 @@
         <v>31</v>
       </c>
       <c r="B25" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D25" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E25" t="b">
         <v>0</v>
@@ -1342,13 +1339,13 @@
         <v>32</v>
       </c>
       <c r="B26" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D26" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E26" t="b">
         <v>0</v>
@@ -1368,13 +1365,13 @@
         <v>33</v>
       </c>
       <c r="B27" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C27" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D27" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E27" t="b">
         <v>0</v>
@@ -1394,13 +1391,13 @@
         <v>34</v>
       </c>
       <c r="B28" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D28" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E28" t="b">
         <v>0</v>
@@ -1420,13 +1417,13 @@
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D29" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E29" t="b">
         <v>0</v>
@@ -1446,13 +1443,13 @@
         <v>36</v>
       </c>
       <c r="B30" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C30" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E30" t="b">
         <v>0</v>
@@ -1472,13 +1469,13 @@
         <v>37</v>
       </c>
       <c r="B31" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C31" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E31" t="b">
         <v>0</v>
@@ -1498,13 +1495,13 @@
         <v>38</v>
       </c>
       <c r="B32" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C32" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D32" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E32" t="b">
         <v>0</v>
@@ -1524,13 +1521,13 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C33" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D33" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E33" t="b">
         <v>0</v>
@@ -1550,13 +1547,13 @@
         <v>40</v>
       </c>
       <c r="B34" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C34" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D34" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E34" t="b">
         <v>0</v>
@@ -1576,13 +1573,13 @@
         <v>41</v>
       </c>
       <c r="B35" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C35" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D35" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E35" t="b">
         <v>0</v>
@@ -1602,13 +1599,13 @@
         <v>42</v>
       </c>
       <c r="B36" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C36" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D36" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E36" t="b">
         <v>0</v>
@@ -1628,13 +1625,13 @@
         <v>43</v>
       </c>
       <c r="B37" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C37" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E37" t="b">
         <v>0</v>
@@ -1654,13 +1651,13 @@
         <v>44</v>
       </c>
       <c r="B38" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C38" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D38" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E38" t="b">
         <v>0</v>
@@ -1680,13 +1677,13 @@
         <v>8</v>
       </c>
       <c r="B39" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C39" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D39" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E39" t="b">
         <v>0</v>
@@ -1703,13 +1700,13 @@
         <v>45</v>
       </c>
       <c r="B40" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C40" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D40" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
@@ -1726,13 +1723,13 @@
         <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C41" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D41" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E41" t="b">
         <v>0</v>
@@ -1749,13 +1746,13 @@
         <v>47</v>
       </c>
       <c r="B42" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C42" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D42" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
@@ -1772,13 +1769,13 @@
         <v>48</v>
       </c>
       <c r="B43" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C43" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D43" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
@@ -1795,13 +1792,13 @@
         <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C44" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D44" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
@@ -1818,13 +1815,13 @@
         <v>50</v>
       </c>
       <c r="B45" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C45" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D45" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
@@ -1841,13 +1838,13 @@
         <v>51</v>
       </c>
       <c r="B46" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C46" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D46" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E46" t="b">
         <v>0</v>
@@ -1867,13 +1864,13 @@
         <v>52</v>
       </c>
       <c r="B47" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C47" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D47" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E47" t="b">
         <v>0</v>
@@ -1893,13 +1890,13 @@
         <v>53</v>
       </c>
       <c r="B48" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C48" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D48" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E48" t="b">
         <v>0</v>
@@ -1919,13 +1916,13 @@
         <v>54</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C49" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D49" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E49" t="b">
         <v>0</v>
@@ -1945,13 +1942,13 @@
         <v>55</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C50" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D50" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E50" t="b">
         <v>0</v>
@@ -1971,13 +1968,13 @@
         <v>56</v>
       </c>
       <c r="B51" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C51" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D51" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E51" t="b">
         <v>0</v>
@@ -1997,13 +1994,13 @@
         <v>57</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C52" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D52" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E52" t="b">
         <v>0</v>
@@ -2023,10 +2020,10 @@
         <v>58</v>
       </c>
       <c r="B53" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C53" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D53" t="s">
         <v>103</v>
@@ -2035,13 +2032,13 @@
         <v>0</v>
       </c>
       <c r="F53" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H53" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="54" spans="1:8">
@@ -2049,10 +2046,10 @@
         <v>59</v>
       </c>
       <c r="B54" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C54" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D54" t="s">
         <v>103</v>
@@ -2061,13 +2058,13 @@
         <v>0</v>
       </c>
       <c r="F54" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G54" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H54" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:8">
@@ -2075,10 +2072,10 @@
         <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C55" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D55" t="s">
         <v>103</v>
@@ -2087,13 +2084,13 @@
         <v>0</v>
       </c>
       <c r="F55" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H55" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="56" spans="1:8">
@@ -2101,10 +2098,10 @@
         <v>61</v>
       </c>
       <c r="B56" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C56" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D56" t="s">
         <v>103</v>
@@ -2113,13 +2110,13 @@
         <v>0</v>
       </c>
       <c r="F56" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G56" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H56" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="57" spans="1:8">
@@ -2127,10 +2124,10 @@
         <v>62</v>
       </c>
       <c r="B57" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C57" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D57" t="s">
         <v>103</v>
@@ -2139,13 +2136,13 @@
         <v>0</v>
       </c>
       <c r="F57" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G57" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H57" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="58" spans="1:8">
@@ -2153,10 +2150,10 @@
         <v>63</v>
       </c>
       <c r="B58" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C58" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D58" t="s">
         <v>103</v>
@@ -2165,18 +2162,18 @@
         <v>0</v>
       </c>
       <c r="F58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G58" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="H58" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="59" spans="1:8">
       <c r="A59" t="s">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="B59" t="s">
         <v>80</v>
@@ -2185,27 +2182,30 @@
         <v>88</v>
       </c>
       <c r="D59" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E59" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F59" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G59" t="s">
+        <v>110</v>
       </c>
       <c r="H59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="60" spans="1:8">
       <c r="A60" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B60" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C60" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D60" t="s">
         <v>104</v>
@@ -2217,18 +2217,18 @@
         <v>0</v>
       </c>
       <c r="H60" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="61" spans="1:8">
       <c r="A61" t="s">
-        <v>47</v>
+        <v>11</v>
       </c>
       <c r="B61" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C61" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D61" t="s">
         <v>104</v>
@@ -2240,18 +2240,18 @@
         <v>0</v>
       </c>
       <c r="H61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" spans="1:8">
       <c r="A62" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B62" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C62" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D62" t="s">
         <v>104</v>
@@ -2263,21 +2263,21 @@
         <v>0</v>
       </c>
       <c r="H62" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="63" spans="1:8">
       <c r="A63" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="B63" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C63" t="s">
         <v>89</v>
       </c>
       <c r="D63" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E63" t="b">
         <v>1</v>
@@ -2286,7 +2286,7 @@
         <v>0</v>
       </c>
       <c r="H63" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
     </row>
     <row r="64" spans="1:8">
@@ -2294,10 +2294,10 @@
         <v>65</v>
       </c>
       <c r="B64" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C64" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D64" t="s">
         <v>105</v>
@@ -2309,7 +2309,7 @@
         <v>0</v>
       </c>
       <c r="H64" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="65" spans="1:8">
@@ -2317,10 +2317,10 @@
         <v>66</v>
       </c>
       <c r="B65" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C65" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D65" t="s">
         <v>105</v>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="H65" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="66" spans="1:8">
@@ -2340,10 +2340,10 @@
         <v>67</v>
       </c>
       <c r="B66" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C66" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D66" t="s">
         <v>105</v>
@@ -2355,7 +2355,7 @@
         <v>0</v>
       </c>
       <c r="H66" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="67" spans="1:8">
@@ -2363,13 +2363,13 @@
         <v>68</v>
       </c>
       <c r="B67" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C67" t="s">
         <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E67" t="b">
         <v>1</v>
@@ -2378,7 +2378,7 @@
         <v>0</v>
       </c>
       <c r="H67" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="68" spans="1:8">
@@ -2386,10 +2386,10 @@
         <v>69</v>
       </c>
       <c r="B68" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C68" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D68" t="s">
         <v>106</v>
@@ -2401,7 +2401,7 @@
         <v>0</v>
       </c>
       <c r="H68" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" spans="1:8">
@@ -2409,10 +2409,10 @@
         <v>70</v>
       </c>
       <c r="B69" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C69" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D69" t="s">
         <v>106</v>
@@ -2424,7 +2424,7 @@
         <v>0</v>
       </c>
       <c r="H69" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:8">
@@ -2432,10 +2432,10 @@
         <v>71</v>
       </c>
       <c r="B70" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C70" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D70" t="s">
         <v>106</v>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
       <c r="H70" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:8">
@@ -2455,10 +2455,10 @@
         <v>72</v>
       </c>
       <c r="B71" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C71" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D71" t="s">
         <v>106</v>
@@ -2470,7 +2470,7 @@
         <v>0</v>
       </c>
       <c r="H71" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="72" spans="1:8">
@@ -2478,10 +2478,10 @@
         <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C72" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D72" t="s">
         <v>106</v>
@@ -2493,7 +2493,7 @@
         <v>0</v>
       </c>
       <c r="H72" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="73" spans="1:8">
@@ -2501,10 +2501,10 @@
         <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C73" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D73" t="s">
         <v>106</v>
@@ -2516,7 +2516,7 @@
         <v>0</v>
       </c>
       <c r="H73" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74" spans="1:8">
@@ -2524,22 +2524,22 @@
         <v>75</v>
       </c>
       <c r="B74" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C74" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D74" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E74" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F74" t="b">
         <v>0</v>
       </c>
       <c r="H74" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="75" spans="1:8">
@@ -2547,10 +2547,10 @@
         <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C75" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D75" t="s">
         <v>107</v>
@@ -2562,44 +2562,41 @@
         <v>0</v>
       </c>
       <c r="H75" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="76" spans="1:8">
       <c r="A76" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="B76" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C76" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D76" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E76" t="b">
         <v>0</v>
       </c>
       <c r="F76" t="b">
-        <v>1</v>
-      </c>
-      <c r="G76" t="s">
-        <v>110</v>
+        <v>0</v>
       </c>
       <c r="H76" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="77" spans="1:8">
       <c r="A77" t="s">
-        <v>77</v>
+        <v>51</v>
       </c>
       <c r="B77" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C77" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D77" t="s">
         <v>108</v>
@@ -2611,21 +2608,21 @@
         <v>1</v>
       </c>
       <c r="G77" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H77" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="78" spans="1:8">
       <c r="A78" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C78" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D78" t="s">
         <v>108</v>
@@ -2637,21 +2634,21 @@
         <v>1</v>
       </c>
       <c r="G78" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H78" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="79" spans="1:8">
       <c r="A79" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B79" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C79" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
         <v>108</v>
@@ -2663,21 +2660,21 @@
         <v>1</v>
       </c>
       <c r="G79" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H79" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:8">
       <c r="A80" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B80" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C80" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D80" t="s">
         <v>108</v>
@@ -2689,21 +2686,21 @@
         <v>1</v>
       </c>
       <c r="G80" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H80" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="81" spans="1:8">
       <c r="A81" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B81" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C81" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="D81" t="s">
         <v>108</v>
@@ -2715,10 +2712,166 @@
         <v>1</v>
       </c>
       <c r="G81" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H81" t="s">
-        <v>129</v>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
+      <c r="A82" t="s">
+        <v>56</v>
+      </c>
+      <c r="B82" t="s">
+        <v>81</v>
+      </c>
+      <c r="C82" t="s">
+        <v>92</v>
+      </c>
+      <c r="D82" t="s">
+        <v>108</v>
+      </c>
+      <c r="E82" t="b">
+        <v>0</v>
+      </c>
+      <c r="F82" t="b">
+        <v>1</v>
+      </c>
+      <c r="G82" t="s">
+        <v>111</v>
+      </c>
+      <c r="H82" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" t="s">
+        <v>57</v>
+      </c>
+      <c r="B83" t="s">
+        <v>81</v>
+      </c>
+      <c r="C83" t="s">
+        <v>92</v>
+      </c>
+      <c r="D83" t="s">
+        <v>108</v>
+      </c>
+      <c r="E83" t="b">
+        <v>0</v>
+      </c>
+      <c r="F83" t="b">
+        <v>1</v>
+      </c>
+      <c r="G83" t="s">
+        <v>111</v>
+      </c>
+      <c r="H83" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
+      <c r="A84" t="s">
+        <v>58</v>
+      </c>
+      <c r="B84" t="s">
+        <v>81</v>
+      </c>
+      <c r="C84" t="s">
+        <v>92</v>
+      </c>
+      <c r="D84" t="s">
+        <v>108</v>
+      </c>
+      <c r="E84" t="b">
+        <v>0</v>
+      </c>
+      <c r="F84" t="b">
+        <v>1</v>
+      </c>
+      <c r="G84" t="s">
+        <v>111</v>
+      </c>
+      <c r="H84" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
+        <v>59</v>
+      </c>
+      <c r="B85" t="s">
+        <v>81</v>
+      </c>
+      <c r="C85" t="s">
+        <v>92</v>
+      </c>
+      <c r="D85" t="s">
+        <v>108</v>
+      </c>
+      <c r="E85" t="b">
+        <v>0</v>
+      </c>
+      <c r="F85" t="b">
+        <v>1</v>
+      </c>
+      <c r="G85" t="s">
+        <v>111</v>
+      </c>
+      <c r="H85" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
+      <c r="A86" t="s">
+        <v>60</v>
+      </c>
+      <c r="B86" t="s">
+        <v>81</v>
+      </c>
+      <c r="C86" t="s">
+        <v>92</v>
+      </c>
+      <c r="D86" t="s">
+        <v>108</v>
+      </c>
+      <c r="E86" t="b">
+        <v>0</v>
+      </c>
+      <c r="F86" t="b">
+        <v>1</v>
+      </c>
+      <c r="G86" t="s">
+        <v>111</v>
+      </c>
+      <c r="H86" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" t="s">
+        <v>64</v>
+      </c>
+      <c r="B87" t="s">
+        <v>81</v>
+      </c>
+      <c r="C87" t="s">
+        <v>92</v>
+      </c>
+      <c r="D87" t="s">
+        <v>108</v>
+      </c>
+      <c r="E87" t="b">
+        <v>0</v>
+      </c>
+      <c r="F87" t="b">
+        <v>1</v>
+      </c>
+      <c r="G87" t="s">
+        <v>111</v>
+      </c>
+      <c r="H87" t="s">
+        <v>128</v>
       </c>
     </row>
   </sheetData>

</xml_diff>